<commit_message>
Corrida | ARG-PIB | 2026-03-09 09:24:15.257371
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -103,13 +103,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">04/03/2026</t>
+    <t xml:space="preserve">09/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-03-10 10:41:15.045703
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -103,13 +103,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">09/03/2026</t>
+    <t xml:space="preserve">10/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-03-10 11:22:58.673715
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Correlograma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Correlograma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="325">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -899,6 +900,63 @@
   </si>
   <si>
     <t xml:space="preserve">2030T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias de las series incluidas en la hoja Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_normal | serie original con 4 forecasts obtenidos del mejor modelo ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_optimista | serie original con 4 forecasts, intervalo y límite optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_pesimista | serie original con 4 forecasts, intervalo y límite pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_d16 | salida D16 del X13-ARIMA-SEATS con los factores estacionales de la serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_c17 | salida C17 del X13-ARIMA-SEATS con pesos del irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_d12 | salida D12 del X13-ARIMA-SEATS con el componente tendencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_1600 | tendencia HP de largo plazo con un lambda de 1.600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_200 | suavizado con filtro HP usando lambda de 200, sirve para determinar PG automáticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e_ajustada | serie ajustada por estacionalidad usando el mejor modelo (LOG o NIV según el caso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_filtrada | serie ajustada por estacionalidad y corregida por irregularidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final | serie f_filtrada con o sin suavizado 2x2 según el caso (es la vieja española)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final_fct_normal | a_original_fct ajustada por D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_tctl | tasas de cambio trimestral logarítmicas de la serie g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_var_interanual | variaciones interanuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_var_trimestral | variaciones trimestrales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_irregular | g_final/d_d12 componente irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i_dt | g_final/d_hp_1600 desvíos respecto de la tendencia</t>
   </si>
   <si>
     <t xml:space="preserve">Coeficientes de correlación de TCTL del ICA-SFE y serie específica</t>
@@ -15547,6 +15605,112 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>313</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -15555,7 +15719,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -15565,13 +15729,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.00543756979155652</v>
@@ -15579,7 +15743,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.139907470762606</v>
@@ -15587,7 +15751,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.384546133510046</v>
@@ -15595,7 +15759,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.641496500806375</v>
@@ -15603,7 +15767,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.721351108080181</v>
@@ -15611,7 +15775,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.510349514612105</v>
@@ -15619,7 +15783,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.160640808108537</v>
@@ -15627,7 +15791,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-0.0491192693391144</v>
@@ -15635,7 +15799,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>-0.104889571770122</v>

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-03-19 12:06:06.585403
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">10/03/2026</t>
+    <t xml:space="preserve">19/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1523,7 +1523,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.721351108080181</v>
+        <v>0.72114005649416</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1581,7 +1581,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.520347421128504</v>
+        <v>0.520042981080401</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1651,7 +1651,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.185066455903565</v>
+        <v>0.177124125660377</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1681,7 +1681,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000146866307519825</v>
+        <v>0.000155068376420352</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -15738,7 +15738,7 @@
         <v>316</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00543756979155652</v>
+        <v>0.00439937513385089</v>
       </c>
     </row>
     <row r="6">
@@ -15746,7 +15746,7 @@
         <v>317</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.139907470762606</v>
+        <v>0.139183420276649</v>
       </c>
     </row>
     <row r="7">
@@ -15754,7 +15754,7 @@
         <v>318</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.384546133510046</v>
+        <v>0.384914465135252</v>
       </c>
     </row>
     <row r="8">
@@ -15762,7 +15762,7 @@
         <v>319</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.641496500806375</v>
+        <v>0.642044945631027</v>
       </c>
     </row>
     <row r="9">
@@ -15770,7 +15770,7 @@
         <v>320</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.721351108080181</v>
+        <v>0.72114005649416</v>
       </c>
     </row>
     <row r="10">
@@ -15778,7 +15778,7 @@
         <v>321</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.510349514612105</v>
+        <v>0.509907861023004</v>
       </c>
     </row>
     <row r="11">
@@ -15786,7 +15786,7 @@
         <v>322</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.160640808108537</v>
+        <v>0.160309882800666</v>
       </c>
     </row>
     <row r="12">
@@ -15794,7 +15794,7 @@
         <v>323</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0491192693391144</v>
+        <v>-0.0493548644001488</v>
       </c>
     </row>
     <row r="13">
@@ -15802,7 +15802,7 @@
         <v>324</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.104889571770122</v>
+        <v>-0.105263379863882</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-05-08 10:11:49.174947
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">25/03/2026</t>
+    <t xml:space="preserve">08/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1523,7 +1523,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.721251404033602</v>
+        <v>0.721364907978918</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1581,7 +1581,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.520203587820442</v>
+        <v>0.520367330463434</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1651,7 +1651,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.181327766662582</v>
+        <v>0.194861038674566</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1681,7 +1681,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000115221997963427</v>
+        <v>0.00011630343719005</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -15774,7 +15774,7 @@
         <v>316</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.00120555741476047</v>
+        <v>-0.000769078242954611</v>
       </c>
     </row>
     <row r="6">
@@ -15782,7 +15782,7 @@
         <v>317</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.136501784403018</v>
+        <v>0.13657789050616</v>
       </c>
     </row>
     <row r="7">
@@ -15790,7 +15790,7 @@
         <v>318</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.387779855208663</v>
+        <v>0.386399397034226</v>
       </c>
     </row>
     <row r="8">
@@ -15798,7 +15798,7 @@
         <v>319</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.643187517967728</v>
+        <v>0.642797690787341</v>
       </c>
     </row>
     <row r="9">
@@ -15806,7 +15806,7 @@
         <v>320</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.721251404033602</v>
+        <v>0.721364907978918</v>
       </c>
     </row>
     <row r="10">
@@ -15814,7 +15814,7 @@
         <v>321</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.508419114964576</v>
+        <v>0.508228764556184</v>
       </c>
     </row>
     <row r="11">
@@ -15822,7 +15822,7 @@
         <v>322</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.158853811652554</v>
+        <v>0.158934456910895</v>
       </c>
     </row>
     <row r="12">
@@ -15830,7 +15830,7 @@
         <v>323</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0461316885701389</v>
+        <v>-0.045118324356173</v>
       </c>
     </row>
     <row r="13">
@@ -15838,7 +15838,7 @@
         <v>324</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.103003542679269</v>
+        <v>-0.103108260403738</v>
       </c>
     </row>
     <row r="14">
@@ -15896,237 +15896,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB35234A-69CC-4480-B276-0142BF48427D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF26BE08-CA3E-42E6-9D32-0E9E282D00FD}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1156A039-7F4A-404A-AA59-0CFBD3EAAB70}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-05-19 14:24:57.145728
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/05/2026</t>
+    <t xml:space="preserve">19/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1523,7 +1523,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.721364907978918</v>
+        <v>0.717944991240825</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1581,7 +1581,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.520367330463434</v>
+        <v>0.515445010447788</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1651,7 +1651,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.194861038674566</v>
+        <v>0.196647137065288</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1681,7 +1681,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00011630343719005</v>
+        <v>0.000107731607137423</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -15774,7 +15774,7 @@
         <v>316</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.000769078242954611</v>
+        <v>-0.000421437147776817</v>
       </c>
     </row>
     <row r="6">
@@ -15782,7 +15782,7 @@
         <v>317</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.13657789050616</v>
+        <v>0.138775419152784</v>
       </c>
     </row>
     <row r="7">
@@ -15790,7 +15790,7 @@
         <v>318</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.386399397034226</v>
+        <v>0.39200415755766</v>
       </c>
     </row>
     <row r="8">
@@ -15798,7 +15798,7 @@
         <v>319</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.642797690787341</v>
+        <v>0.640616110373754</v>
       </c>
     </row>
     <row r="9">
@@ -15806,7 +15806,7 @@
         <v>320</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.721364907978918</v>
+        <v>0.717944991240825</v>
       </c>
     </row>
     <row r="10">
@@ -15814,7 +15814,7 @@
         <v>321</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.508228764556184</v>
+        <v>0.507527805395759</v>
       </c>
     </row>
     <row r="11">
@@ -15822,7 +15822,7 @@
         <v>322</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.158934456910895</v>
+        <v>0.158390268508302</v>
       </c>
     </row>
     <row r="12">
@@ -15830,7 +15830,7 @@
         <v>323</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.045118324356173</v>
+        <v>-0.0423901973361968</v>
       </c>
     </row>
     <row r="13">
@@ -15838,7 +15838,7 @@
         <v>324</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.103108260403738</v>
+        <v>-0.100590409821635</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Corrida | ARG-PIB | 2026-06-17 10:41:47.580482
</commit_message>
<xml_diff>
--- a/indicadores/ARG-PIB_out.xlsx
+++ b/indicadores/ARG-PIB_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="327">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentina</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">19/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">fleiva</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1491,9 +1497,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1504,7 +1514,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1518,12 +1528,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.717944991240825</v>
+        <v>0.718351631330702</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1534,7 +1544,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1562,7 +1572,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1576,12 +1586,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.515445010447788</v>
+        <v>0.51602906623548</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1604,7 +1614,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1618,7 +1628,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1632,7 +1642,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1646,12 +1656,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.196647137065288</v>
+        <v>0.224264939275511</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1662,7 +1672,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1676,12 +1686,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000107731607137423</v>
+        <v>0.0000792883206407128</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1824,10 +1834,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1840,10 +1850,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1867,66 +1877,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>274720.736810153</v>
@@ -1979,7 +1989,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>293673.715991951</v>
@@ -2036,7 +2046,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>286997.615166001</v>
@@ -2093,7 +2103,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>284846.968573894</v>
@@ -2150,7 +2160,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>279343.652369923</v>
@@ -2209,7 +2219,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>307042.161198174</v>
@@ -2268,7 +2278,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>299264.747389256</v>
@@ -2327,7 +2337,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>297477.956413941</v>
@@ -2386,7 +2396,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>286838.428333654</v>
@@ -2445,7 +2455,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>303299.646282604</v>
@@ -2504,7 +2514,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>306691.300424839</v>
@@ -2563,7 +2573,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>310878.888728805</v>
@@ -2622,7 +2632,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>297656.635511472</v>
@@ -2681,7 +2691,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>316177.536148331</v>
@@ -2740,7 +2750,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>311431.169575721</v>
@@ -2799,7 +2809,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>327668.22647504</v>
@@ -2858,7 +2868,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>317571.233109077</v>
@@ -2917,7 +2927,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>336774.36302742</v>
@@ -2976,7 +2986,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>328317.968647882</v>
@@ -3035,7 +3045,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>338005.624444955</v>
@@ -3094,7 +3104,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>322824.398576504</v>
@@ -3153,7 +3163,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>337794.458238781</v>
@@ -3212,7 +3222,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>322171.407692798</v>
@@ -3271,7 +3281,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>330046.282827642</v>
@@ -3330,7 +3340,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>319289.801156244</v>
@@ -3389,7 +3399,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>328954.715977267</v>
@@ -3448,7 +3458,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>329916.334393073</v>
@@ -3507,7 +3517,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>334516.508976794</v>
@@ -3566,7 +3576,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>333324.232089629</v>
@@ -3625,7 +3635,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>354687.754732671</v>
@@ -3684,7 +3694,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>361155.938063312</v>
@@ -3743,7 +3753,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>347326.175914372</v>
@@ -3802,7 +3812,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>317805.1402913</v>
@@ -3861,7 +3871,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>336329.289639023</v>
@@ -3920,7 +3930,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>345471.162010909</v>
@@ -3979,7 +3989,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>351893.863389451</v>
@@ -4038,7 +4048,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>344733.704644733</v>
@@ -4097,7 +4107,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>365460.47995839</v>
@@ -4156,7 +4166,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>363105.164581838</v>
@@ -4215,7 +4225,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>373039.722404591</v>
@@ -4274,7 +4284,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>350886.763021546</v>
@@ -4333,7 +4343,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>375630.182793721</v>
@@ -4392,7 +4402,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>392787.639412916</v>
@@ -4451,7 +4461,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>387175.795813475</v>
@@ -4510,7 +4520,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>348787.74219593</v>
@@ -4569,7 +4579,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>365764.156070867</v>
@@ -4628,7 +4638,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>356438.374654421</v>
@@ -4687,7 +4697,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>353808.753269303</v>
@@ -4746,7 +4756,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>326438.28846154</v>
@@ -4805,7 +4815,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>336012.476528146</v>
@@ -4864,7 +4874,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>355257.567292421</v>
@@ -4923,7 +4933,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>362089.394512038</v>
@@ -4982,7 +4992,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>335280.801750139</v>
@@ -5041,7 +5051,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>361986.010937587</v>
@@ -5100,7 +5110,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>371728.866385673</v>
@@ -5159,7 +5169,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>367537.47434082</v>
@@ -5218,7 +5228,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>335440.414960448</v>
@@ -5277,7 +5287,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>372878.925634586</v>
@@ -5336,7 +5346,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>377126.467131091</v>
@@ -5395,7 +5405,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>379809.195369898</v>
@@ -5454,7 +5464,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>327369.620852271</v>
@@ -5513,7 +5523,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>342983.11820777</v>
@@ -5572,7 +5582,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>338381.469087693</v>
@@ -5631,7 +5641,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>354683.615755327</v>
@@ -5690,7 +5700,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>330021.402388751</v>
@@ -5749,7 +5759,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>367750.910840104</v>
@@ -5808,7 +5818,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>385564.691568936</v>
@@ -5867,7 +5877,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>377396.585608765</v>
@@ -5926,7 +5936,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>342518.805916862</v>
@@ -5985,7 +5995,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>384165.470300204</v>
@@ -6044,7 +6054,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>394585.944646856</v>
@@ -6103,7 +6113,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>377308.717854857</v>
@@ -6162,7 +6172,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>358624.233714962</v>
@@ -6221,7 +6231,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>379121.886615641</v>
@@ -6280,7 +6290,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>367102.679295591</v>
@@ -6339,7 +6349,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>365343.872206465</v>
@@ -6398,7 +6408,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>344056.129030727</v>
@@ -6457,7 +6467,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>344664.833564317</v>
@@ -6516,7 +6526,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>330724.443386007</v>
@@ -6575,7 +6585,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>348765.952516928</v>
@@ -6634,7 +6644,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>300955.694107537</v>
@@ -6693,7 +6703,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>333959.889781522</v>
@@ -6752,7 +6762,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>348762.379985619</v>
@@ -6811,7 +6821,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>359489.605138886</v>
@@ -6870,7 +6880,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>325091.525804152</v>
@@ -6929,7 +6939,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>376116.498579129</v>
@@ -6988,7 +6998,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>384748.078172234</v>
@@ -7047,7 +7057,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>399299.25475537</v>
@@ -7106,7 +7116,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>372951.254774255</v>
@@ -7165,7 +7175,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>421992.062398688</v>
@@ -7224,7 +7234,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>418269.85525714</v>
@@ -7283,7 +7293,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>414719.066729715</v>
@@ -7342,7 +7352,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>390107.470249262</v>
@@ -7401,7 +7411,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>436086.196210652</v>
@@ -7460,7 +7470,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>437481.084266889</v>
@@ -7519,7 +7529,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>441964.886493292</v>
@@ -7578,7 +7588,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>419991.981226533</v>
@@ -7637,7 +7647,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>464221.511045238</v>
@@ -7696,7 +7706,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>456993.219112459</v>
@@ -7755,7 +7765,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>463977.478231814</v>
@@ -7814,7 +7824,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>429047.866823909</v>
@@ -7873,7 +7883,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>447303.84163999</v>
@@ -7932,7 +7942,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>436704.325551312</v>
@@ -7991,7 +8001,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>440766.881538129</v>
@@ -8050,7 +8060,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>426519.991695787</v>
@@ -8109,7 +8119,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>470126.272390857</v>
@@ -8168,7 +8178,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>472677.535758481</v>
@@ -8227,7 +8237,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>481427.468387569</v>
@@ -8286,7 +8296,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>462258.015087104</v>
@@ -8345,7 +8355,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>508020.740483857</v>
@@ -8404,7 +8414,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>512208.063825329</v>
@@ -8463,7 +8473,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>518379.749569641</v>
@@ -8522,7 +8532,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>489869.523456675</v>
@@ -8581,7 +8591,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>543066.384243079</v>
@@ -8640,7 +8650,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>528837.044115363</v>
@@ -8699,7 +8709,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>516130.558988705</v>
@@ -8758,7 +8768,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>477829.815015122</v>
@@ -8817,7 +8827,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>516391.046914062</v>
@@ -8876,7 +8886,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>502076.175540002</v>
@@ -8935,7 +8945,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>511259.942382052</v>
@@ -8994,7 +9004,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>476984.733765134</v>
@@ -9053,7 +9063,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>514340.804852638</v>
@@ -9112,7 +9122,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>499002.622761819</v>
@@ -9171,7 +9181,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>501389.215538927</v>
@@ -9230,7 +9240,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>467327.980201225</v>
@@ -9289,7 +9299,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>513476.440667766</v>
@@ -9348,7 +9358,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>474407.554522122</v>
@@ -9407,7 +9417,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>448693.775149267</v>
@@ -9466,7 +9476,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>390971.781617488</v>
@@ -9525,7 +9535,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>444096.358125271</v>
@@ -9584,7 +9594,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>428054.007663138</v>
@@ -9643,7 +9653,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>433362.880156828</v>
@@ -9702,7 +9712,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>412150.09254573</v>
@@ -9761,7 +9771,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>478511.050017991</v>
@@ -9820,7 +9830,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>471537.267275214</v>
@@ -9879,7 +9889,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>484205.691494541</v>
@@ -9938,7 +9948,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>460369.442232949</v>
@@ -9997,7 +10007,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>514395.681772362</v>
@@ -10056,7 +10066,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>481151.979943508</v>
@@ -10115,7 +10125,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>484543.676876562</v>
@@ -10174,7 +10184,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>493602.530577855</v>
@@ -10233,7 +10243,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>581668.249879602</v>
@@ -10292,7 +10302,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>514697.789505428</v>
@@ -10351,7 +10361,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>522255.200050771</v>
@@ -10410,7 +10420,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>532348.212016917</v>
@@ -10469,7 +10479,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>614076.392608544</v>
@@ -10528,7 +10538,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>562978.965626877</v>
@@ -10587,7 +10597,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>572794.046630588</v>
@@ -10646,7 +10656,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>576846.885699427</v>
@@ -10705,7 +10715,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>674620.563006485</v>
@@ -10764,7 +10774,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>610425.694014854</v>
@@ -10823,7 +10833,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>625876.867863597</v>
@@ -10882,7 +10892,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>616720.357064478</v>
@@ -10941,7 +10951,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>711405.500455233</v>
@@ -11000,7 +11010,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>647087.959742494</v>
@@ -11059,7 +11069,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>613490.821702641</v>
@@ -11118,7 +11128,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>578553.044242405</v>
@@ -11177,7 +11187,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>631197.751860069</v>
@@ -11236,7 +11246,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>610519.854611727</v>
@@ -11295,7 +11305,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>615220.854937297</v>
@@ -11354,7 +11364,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>611607.33658973</v>
@@ -11413,7 +11423,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>733730.773968903</v>
@@ -11472,7 +11482,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>668566.509488986</v>
@@ -11531,7 +11541,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>668190.097719574</v>
@@ -11590,7 +11600,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>662325.585972695</v>
@@ -11649,7 +11659,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>766332.954571613</v>
@@ -11708,7 +11718,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>711417.391930105</v>
@@ -11767,7 +11777,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>703050.456407993</v>
@@ -11826,7 +11836,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>672685.993630504</v>
@@ -11885,7 +11895,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>730838.272592776</v>
@@ -11944,7 +11954,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>703461.652530196</v>
@@ -12003,7 +12013,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>706958.039082319</v>
@@ -12062,7 +12072,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>677085.529173151</v>
@@ -12121,7 +12131,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>776486.60279942</v>
@@ -12180,7 +12190,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>721458.944216182</v>
@@ -12239,7 +12249,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>706597.345022507</v>
@@ -12298,7 +12308,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>671066.046635063</v>
@@ -12357,7 +12367,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>760576.868348004</v>
@@ -12416,7 +12426,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>690879.798251683</v>
@@ -12475,7 +12485,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>686701.470618711</v>
@@ -12534,7 +12544,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>672749.811391699</v>
@@ -12593,7 +12603,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>791235.96554167</v>
@@ -12652,7 +12662,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>718281.265449782</v>
@@ -12711,7 +12721,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>703681.544169008</v>
@@ -12770,7 +12780,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>677652.089115703</v>
@@ -12829,7 +12839,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>760703.280151656</v>
@@ -12888,7 +12898,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>694382.47577623</v>
@@ -12947,7 +12957,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>693173.549347058</v>
@@ -13006,7 +13016,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>681444.766110222</v>
@@ -13065,7 +13075,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>778401.676449317</v>
@@ -13124,7 +13134,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>721120.426852794</v>
@@ -13183,7 +13193,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>724592.921638963</v>
@@ -13242,7 +13252,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>707324.268057214</v>
@@ -13301,7 +13311,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>747428.299954575</v>
@@ -13360,7 +13370,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>696101.583521808</v>
@@ -13419,7 +13429,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>678655.620384454</v>
@@ -13478,7 +13488,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>665848.715299709</v>
@@ -13537,7 +13547,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>751784.460777133</v>
@@ -13596,7 +13606,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>683900.898552578</v>
@@ -13655,7 +13665,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>671361.13972242</v>
@@ -13714,7 +13724,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>632389.35353461</v>
@@ -13773,7 +13783,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>609379.989464801</v>
@@ -13832,7 +13842,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>614192.478404223</v>
@@ -13891,7 +13901,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>642403.32319795</v>
@@ -13950,7 +13960,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>652831.976706322</v>
@@ -14009,7 +14019,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>723516.622490675</v>
@@ -14068,7 +14078,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>686756.467826674</v>
@@ -14127,7 +14137,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>696134.669112115</v>
@@ -14186,7 +14196,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>697625.284666358</v>
@@ -14245,7 +14255,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>782338.628533735</v>
@@ -14304,7 +14314,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>732662.163875501</v>
@@ -14363,7 +14373,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>712740.457828738</v>
@@ -14422,7 +14432,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>703987.504321577</v>
@@ -14481,7 +14491,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>737941.909374072</v>
@@ -14540,7 +14550,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>728638.584568682</v>
@@ -14599,7 +14609,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>700509.934572323</v>
@@ -14658,7 +14668,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>669057.733385167</v>
@@ -14717,7 +14727,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>729947.785274553</v>
@@ -14776,7 +14786,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>714524.365549959</v>
@@ -14835,7 +14845,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>718991.46093658</v>
@@ -14894,7 +14904,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>708113.805670176</v>
@@ -14953,7 +14963,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>776528.776090785</v>
@@ -15012,7 +15022,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>737795.741613431</v>
@@ -15071,7 +15081,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>733788.66978506</v>
@@ -15130,7 +15140,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2"/>
       <c r="C226" s="3" t="n">
@@ -15163,7 +15173,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="3" t="n">
@@ -15196,7 +15206,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2"/>
       <c r="C228" s="3" t="n">
@@ -15229,7 +15239,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2"/>
       <c r="C229" s="3" t="n">
@@ -15262,7 +15272,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2"/>
       <c r="C230" s="3"/>
@@ -15285,7 +15295,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2"/>
       <c r="C231" s="3"/>
@@ -15308,7 +15318,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2"/>
       <c r="C232" s="3"/>
@@ -15331,7 +15341,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2"/>
       <c r="C233" s="3"/>
@@ -15354,7 +15364,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2"/>
       <c r="C234" s="3"/>
@@ -15377,7 +15387,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2"/>
       <c r="C235" s="3"/>
@@ -15400,7 +15410,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2"/>
       <c r="C236" s="3"/>
@@ -15423,7 +15433,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2"/>
       <c r="C237" s="3"/>
@@ -15446,7 +15456,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2"/>
       <c r="C238" s="3"/>
@@ -15469,7 +15479,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="3"/>
@@ -15492,7 +15502,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2"/>
       <c r="C240" s="3"/>
@@ -15515,7 +15525,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2"/>
       <c r="C241" s="3"/>
@@ -15538,7 +15548,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2"/>
       <c r="C242" s="3"/>
@@ -15561,7 +15571,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2"/>
       <c r="C243" s="3"/>
@@ -15584,7 +15594,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2"/>
       <c r="C244" s="3"/>
@@ -15607,7 +15617,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2"/>
       <c r="C245" s="3"/>
@@ -15641,97 +15651,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -15755,7 +15765,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -15765,80 +15775,80 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.000421437147776817</v>
+        <v>-0.000167205647467741</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.138775419152784</v>
+        <v>0.140096868939759</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.39200415755766</v>
+        <v>0.391439422807531</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.640616110373754</v>
+        <v>0.639736075454993</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.717944991240825</v>
+        <v>0.718351631330702</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.507527805395759</v>
+        <v>0.509737771049973</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.158390268508302</v>
+        <v>0.160042663783679</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0423901973361968</v>
+        <v>-0.0424877196871654</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>-0.100590409821635</v>
+        <v>-0.100533429495466</v>
       </c>
     </row>
     <row r="14">

</xml_diff>